<commit_message>
Update code, figures, source_data; ignore *.zip
</commit_message>
<xml_diff>
--- a/source_data/Fig2_source_data.xlsx
+++ b/source_data/Fig2_source_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="3172" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="3700" uniqueCount="14">
   <si>
     <t>r_a0_fapar</t>
   </si>
@@ -2224,7 +2224,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1579"/>
+  <dimension ref="A1:D1842"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.453125" customWidth="true"/>
@@ -24327,6 +24327,3686 @@
         <v>0.62797220774122797</v>
       </c>
     </row>
+    <row r="1580">
+      <c r="A1580" s="0">
+        <v>51.307609999999997</v>
+      </c>
+      <c r="B1580" s="0">
+        <v>4.5198400000000003</v>
+      </c>
+      <c r="C1580" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1580" s="0">
+        <v>0.72826254976572802</v>
+      </c>
+    </row>
+    <row r="1581">
+      <c r="A1581" s="0">
+        <v>50.311875999999998</v>
+      </c>
+      <c r="B1581" s="0">
+        <v>4.9681129999999998</v>
+      </c>
+      <c r="C1581" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1581" s="0">
+        <v>0.81808581510645095</v>
+      </c>
+    </row>
+    <row r="1582">
+      <c r="A1582" s="0">
+        <v>51.112180000000002</v>
+      </c>
+      <c r="B1582" s="0">
+        <v>3.8504299999999998</v>
+      </c>
+      <c r="C1582" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1582" s="0">
+        <v>0.67906827168282602</v>
+      </c>
+    </row>
+    <row r="1583">
+      <c r="A1583" s="0">
+        <v>50.979868000000003</v>
+      </c>
+      <c r="B1583" s="0">
+        <v>5.6318510000000002</v>
+      </c>
+      <c r="C1583" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1583" s="0">
+        <v>0.71667156519452402</v>
+      </c>
+    </row>
+    <row r="1584">
+      <c r="A1584" s="0">
+        <v>50.304962000000003</v>
+      </c>
+      <c r="B1584" s="0">
+        <v>5.9980989999999999</v>
+      </c>
+      <c r="C1584" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1584" s="0">
+        <v>0.71109790234997405</v>
+      </c>
+    </row>
+    <row r="1585">
+      <c r="A1585" s="0">
+        <v>46.583193999999999</v>
+      </c>
+      <c r="B1585" s="0">
+        <v>9.7904169999999997</v>
+      </c>
+      <c r="C1585" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1585" s="0">
+        <v>0.63941448071464002</v>
+      </c>
+    </row>
+    <row r="1586">
+      <c r="A1586" s="0">
+        <v>47.210222219999999</v>
+      </c>
+      <c r="B1586" s="0">
+        <v>8.4104444439999995</v>
+      </c>
+      <c r="C1586" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1586" s="0">
+        <v>0.67575835730911604</v>
+      </c>
+    </row>
+    <row r="1587">
+      <c r="A1587" s="0">
+        <v>46.815330000000003</v>
+      </c>
+      <c r="B1587" s="0">
+        <v>9.8559099999999997</v>
+      </c>
+      <c r="C1587" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1587" s="0">
+        <v>0.80923756721391704</v>
+      </c>
+    </row>
+    <row r="1588">
+      <c r="A1588" s="0">
+        <v>47.115833330000001</v>
+      </c>
+      <c r="B1588" s="0">
+        <v>8.5377777780000006</v>
+      </c>
+      <c r="C1588" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1588" s="0">
+        <v>0.76719528471734999</v>
+      </c>
+    </row>
+    <row r="1589">
+      <c r="A1589" s="0">
+        <v>47.478332999999999</v>
+      </c>
+      <c r="B1589" s="0">
+        <v>8.3643889999999992</v>
+      </c>
+      <c r="C1589" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1589" s="0">
+        <v>0.82491062221012901</v>
+      </c>
+    </row>
+    <row r="1590">
+      <c r="A1590" s="0">
+        <v>49.502076150000001</v>
+      </c>
+      <c r="B1590" s="0">
+        <v>18.536882469999998</v>
+      </c>
+      <c r="C1590" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1590" s="0">
+        <v>0.75016083701220804</v>
+      </c>
+    </row>
+    <row r="1591">
+      <c r="A1591" s="0">
+        <v>48.681548300000003</v>
+      </c>
+      <c r="B1591" s="0">
+        <v>16.946331700000002</v>
+      </c>
+      <c r="C1591" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1591" s="0">
+        <v>0.80498295107907503</v>
+      </c>
+    </row>
+    <row r="1592">
+      <c r="A1592" s="0">
+        <v>49.443723599999999</v>
+      </c>
+      <c r="B1592" s="0">
+        <v>16.696512500000001</v>
+      </c>
+      <c r="C1592" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1592" s="0">
+        <v>0.78097405289133703</v>
+      </c>
+    </row>
+    <row r="1593">
+      <c r="A1593" s="0">
+        <v>49.035975000000001</v>
+      </c>
+      <c r="B1593" s="0">
+        <v>17.969899999999999</v>
+      </c>
+      <c r="C1593" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1593" s="0">
+        <v>0.80730061903824602</v>
+      </c>
+    </row>
+    <row r="1594">
+      <c r="A1594" s="0">
+        <v>49.024650000000001</v>
+      </c>
+      <c r="B1594" s="0">
+        <v>14.770350000000001</v>
+      </c>
+      <c r="C1594" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1594" s="0">
+        <v>0.80135980784922301</v>
+      </c>
+    </row>
+    <row r="1595">
+      <c r="A1595" s="0">
+        <v>53.866169999999997</v>
+      </c>
+      <c r="B1595" s="0">
+        <v>13.68342</v>
+      </c>
+      <c r="C1595" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1595" s="0">
+        <v>0.82908679005672004</v>
+      </c>
+    </row>
+    <row r="1596">
+      <c r="A1596" s="0">
+        <v>50.950040000000001</v>
+      </c>
+      <c r="B1596" s="0">
+        <v>13.512589999999999</v>
+      </c>
+      <c r="C1596" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1596" s="0">
+        <v>0.79247914939298203</v>
+      </c>
+    </row>
+    <row r="1597">
+      <c r="A1597" s="0">
+        <v>51.079408399999998</v>
+      </c>
+      <c r="B1597" s="0">
+        <v>10.4520894</v>
+      </c>
+      <c r="C1597" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1597" s="0">
+        <v>0.76779185981440101</v>
+      </c>
+    </row>
+    <row r="1598">
+      <c r="A1598" s="0">
+        <v>52.086559999999999</v>
+      </c>
+      <c r="B1598" s="0">
+        <v>11.22235</v>
+      </c>
+      <c r="C1598" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1598" s="0">
+        <v>0.70768162255304501</v>
+      </c>
+    </row>
+    <row r="1599">
+      <c r="A1599" s="0">
+        <v>50.963810000000002</v>
+      </c>
+      <c r="B1599" s="0">
+        <v>13.48978</v>
+      </c>
+      <c r="C1599" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1599" s="0">
+        <v>0.78980464212175605</v>
+      </c>
+    </row>
+    <row r="1600">
+      <c r="A1600" s="0">
+        <v>50.786659999999998</v>
+      </c>
+      <c r="B1600" s="0">
+        <v>13.72129</v>
+      </c>
+      <c r="C1600" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1600" s="0">
+        <v>0.78994512655503402</v>
+      </c>
+    </row>
+    <row r="1601">
+      <c r="A1601" s="0">
+        <v>50.621914199999999</v>
+      </c>
+      <c r="B1601" s="0">
+        <v>6.3041255999999999</v>
+      </c>
+      <c r="C1601" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1601" s="0">
+        <v>0.77669386301346</v>
+      </c>
+    </row>
+    <row r="1602">
+      <c r="A1602" s="0">
+        <v>50.504926849999997</v>
+      </c>
+      <c r="B1602" s="0">
+        <v>6.3309624749999998</v>
+      </c>
+      <c r="C1602" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1602" s="0">
+        <v>0.809746626491187</v>
+      </c>
+    </row>
+    <row r="1603">
+      <c r="A1603" s="0">
+        <v>50.962560000000004</v>
+      </c>
+      <c r="B1603" s="0">
+        <v>13.565149999999999</v>
+      </c>
+      <c r="C1603" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1603" s="0">
+        <v>0.82173525444902795</v>
+      </c>
+    </row>
+    <row r="1604">
+      <c r="A1604" s="0">
+        <v>56.073700000000002</v>
+      </c>
+      <c r="B1604" s="0">
+        <v>9.3340999999999994</v>
+      </c>
+      <c r="C1604" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1604" s="0">
+        <v>0.75554737615137901</v>
+      </c>
+    </row>
+    <row r="1605">
+      <c r="A1605" s="0">
+        <v>55.485869399999999</v>
+      </c>
+      <c r="B1605" s="0">
+        <v>11.644644400000001</v>
+      </c>
+      <c r="C1605" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1605" s="0">
+        <v>0.74014986599312205</v>
+      </c>
+    </row>
+    <row r="1606">
+      <c r="A1606" s="0">
+        <v>38.701839</v>
+      </c>
+      <c r="B1606" s="0">
+        <v>-6.7858809999999998</v>
+      </c>
+      <c r="C1606" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1606" s="0">
+        <v>0.67705847878874503</v>
+      </c>
+    </row>
+    <row r="1607">
+      <c r="A1607" s="0">
+        <v>36.940046000000002</v>
+      </c>
+      <c r="B1607" s="0">
+        <v>-2.0332080000000001</v>
+      </c>
+      <c r="C1607" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1607" s="0">
+        <v>0.41817341190132501</v>
+      </c>
+    </row>
+    <row r="1608">
+      <c r="A1608" s="0">
+        <v>36.926594000000001</v>
+      </c>
+      <c r="B1608" s="0">
+        <v>-2.7521149999999999</v>
+      </c>
+      <c r="C1608" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1608" s="0">
+        <v>0.69455760234317898</v>
+      </c>
+    </row>
+    <row r="1609">
+      <c r="A1609" s="0">
+        <v>39.942689999999999</v>
+      </c>
+      <c r="B1609" s="0">
+        <v>-5.778683</v>
+      </c>
+      <c r="C1609" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1609" s="0">
+        <v>0.33461551045427801</v>
+      </c>
+    </row>
+    <row r="1610">
+      <c r="A1610" s="0">
+        <v>39.934592000000002</v>
+      </c>
+      <c r="B1610" s="0">
+        <v>-5.775881</v>
+      </c>
+      <c r="C1610" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1610" s="0">
+        <v>0.35685659340541798</v>
+      </c>
+    </row>
+    <row r="1611">
+      <c r="A1611" s="0">
+        <v>61.847410000000004</v>
+      </c>
+      <c r="B1611" s="0">
+        <v>24.29477</v>
+      </c>
+      <c r="C1611" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1611" s="0">
+        <v>0.79597168492695003</v>
+      </c>
+    </row>
+    <row r="1612">
+      <c r="A1612" s="0">
+        <v>67.987214719999997</v>
+      </c>
+      <c r="B1612" s="0">
+        <v>24.24301028</v>
+      </c>
+      <c r="C1612" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1612" s="0">
+        <v>0.753610728107731</v>
+      </c>
+    </row>
+    <row r="1613">
+      <c r="A1613" s="0">
+        <v>60.641829999999999</v>
+      </c>
+      <c r="B1613" s="0">
+        <v>23.959520000000001</v>
+      </c>
+      <c r="C1613" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1613" s="0">
+        <v>0.79478452926130605</v>
+      </c>
+    </row>
+    <row r="1614">
+      <c r="A1614" s="0">
+        <v>61.832650000000001</v>
+      </c>
+      <c r="B1614" s="0">
+        <v>24.19285</v>
+      </c>
+      <c r="C1614" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1614" s="0">
+        <v>0.74900042412595302</v>
+      </c>
+    </row>
+    <row r="1615">
+      <c r="A1615" s="0">
+        <v>67.754900000000006</v>
+      </c>
+      <c r="B1615" s="0">
+        <v>29.61</v>
+      </c>
+      <c r="C1615" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1615" s="0">
+        <v>0.72288330990301497</v>
+      </c>
+    </row>
+    <row r="1616">
+      <c r="A1616" s="0">
+        <v>44.493653000000002</v>
+      </c>
+      <c r="B1616" s="0">
+        <v>-0.95609200000000005</v>
+      </c>
+      <c r="C1616" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1616" s="0">
+        <v>0.76612528238121402</v>
+      </c>
+    </row>
+    <row r="1617">
+      <c r="A1617" s="0">
+        <v>43.240789999999997</v>
+      </c>
+      <c r="B1617" s="0">
+        <v>5.6786500000000002</v>
+      </c>
+      <c r="C1617" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1617" s="0">
+        <v>0.422278531751829</v>
+      </c>
+    </row>
+    <row r="1618">
+      <c r="A1618" s="0">
+        <v>48.476357999999998</v>
+      </c>
+      <c r="B1618" s="0">
+        <v>2.7800959999999999</v>
+      </c>
+      <c r="C1618" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1618" s="0">
+        <v>0.78456787014143703</v>
+      </c>
+    </row>
+    <row r="1619">
+      <c r="A1619" s="0">
+        <v>48.674100000000003</v>
+      </c>
+      <c r="B1619" s="0">
+        <v>7.0646500000000003</v>
+      </c>
+      <c r="C1619" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1619" s="0">
+        <v>0.825939653277317</v>
+      </c>
+    </row>
+    <row r="1620">
+      <c r="A1620" s="0">
+        <v>47.322916999999997</v>
+      </c>
+      <c r="B1620" s="0">
+        <v>2.2841019999999999</v>
+      </c>
+      <c r="C1620" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1620" s="0">
+        <v>0.78385540120696295</v>
+      </c>
+    </row>
+    <row r="1621">
+      <c r="A1621" s="0">
+        <v>43.572854999999997</v>
+      </c>
+      <c r="B1621" s="0">
+        <v>1.3747400000000001</v>
+      </c>
+      <c r="C1621" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1621" s="0">
+        <v>0.86042545594425302</v>
+      </c>
+    </row>
+    <row r="1622">
+      <c r="A1622" s="0">
+        <v>31.345044590000001</v>
+      </c>
+      <c r="B1622" s="0">
+        <v>35.051988510000001</v>
+      </c>
+      <c r="C1622" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1622" s="0">
+        <v>0.56482099149986198</v>
+      </c>
+    </row>
+    <row r="1623">
+      <c r="A1623" s="0">
+        <v>45.197755000000001</v>
+      </c>
+      <c r="B1623" s="0">
+        <v>10.741966</v>
+      </c>
+      <c r="C1623" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1623" s="0">
+        <v>0.59884591009601396</v>
+      </c>
+    </row>
+    <row r="1624">
+      <c r="A1624" s="0">
+        <v>41.704265589999999</v>
+      </c>
+      <c r="B1624" s="0">
+        <v>12.35729313</v>
+      </c>
+      <c r="C1624" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1624" s="0">
+        <v>0.445903878686848</v>
+      </c>
+    </row>
+    <row r="1625">
+      <c r="A1625" s="0">
+        <v>45.956200000000003</v>
+      </c>
+      <c r="B1625" s="0">
+        <v>11.281319999999999</v>
+      </c>
+      <c r="C1625" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1625" s="0">
+        <v>0.86068326914851601</v>
+      </c>
+    </row>
+    <row r="1626">
+      <c r="A1626" s="0">
+        <v>45.740481000000003</v>
+      </c>
+      <c r="B1626" s="0">
+        <v>12.750297</v>
+      </c>
+      <c r="C1626" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1626" s="0">
+        <v>0.56026668906156796</v>
+      </c>
+    </row>
+    <row r="1627">
+      <c r="A1627" s="0">
+        <v>46.014678000000004</v>
+      </c>
+      <c r="B1627" s="0">
+        <v>11.045831</v>
+      </c>
+      <c r="C1627" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1627" s="0">
+        <v>0.85305867996035401</v>
+      </c>
+    </row>
+    <row r="1628">
+      <c r="A1628" s="0">
+        <v>46.586860000000001</v>
+      </c>
+      <c r="B1628" s="0">
+        <v>11.43369</v>
+      </c>
+      <c r="C1628" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1628" s="0">
+        <v>0.76456186629404199</v>
+      </c>
+    </row>
+    <row r="1629">
+      <c r="A1629" s="0">
+        <v>43.732022000000001</v>
+      </c>
+      <c r="B1629" s="0">
+        <v>10.29091</v>
+      </c>
+      <c r="C1629" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1629" s="0">
+        <v>0.60637451440622003</v>
+      </c>
+    </row>
+    <row r="1630">
+      <c r="A1630" s="0">
+        <v>45.844439999999999</v>
+      </c>
+      <c r="B1630" s="0">
+        <v>7.578055</v>
+      </c>
+      <c r="C1630" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1630" s="0">
+        <v>0.88428004297921903</v>
+      </c>
+    </row>
+    <row r="1631">
+      <c r="A1631" s="0">
+        <v>56.447603000000001</v>
+      </c>
+      <c r="B1631" s="0">
+        <v>32.901878000000004</v>
+      </c>
+      <c r="C1631" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1631" s="0">
+        <v>0.86947117745449398</v>
+      </c>
+    </row>
+    <row r="1632">
+      <c r="A1632" s="0">
+        <v>56.461527799999999</v>
+      </c>
+      <c r="B1632" s="0">
+        <v>32.922083299999997</v>
+      </c>
+      <c r="C1632" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1632" s="0">
+        <v>0.83927158288647297</v>
+      </c>
+    </row>
+    <row r="1633">
+      <c r="A1633" s="0">
+        <v>64.182029</v>
+      </c>
+      <c r="B1633" s="0">
+        <v>19.556539000000001</v>
+      </c>
+      <c r="C1633" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1633" s="0">
+        <v>0.78359449544401405</v>
+      </c>
+    </row>
+    <row r="1634">
+      <c r="A1634" s="0">
+        <v>56.097630000000002</v>
+      </c>
+      <c r="B1634" s="0">
+        <v>13.41897</v>
+      </c>
+      <c r="C1634" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1634" s="0">
+        <v>0.767499207615295</v>
+      </c>
+    </row>
+    <row r="1635">
+      <c r="A1635" s="0">
+        <v>60.086497219999998</v>
+      </c>
+      <c r="B1635" s="0">
+        <v>17.479502780000001</v>
+      </c>
+      <c r="C1635" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1635" s="0">
+        <v>0.76162705083330595</v>
+      </c>
+    </row>
+    <row r="1636">
+      <c r="A1636" s="0">
+        <v>64.1725</v>
+      </c>
+      <c r="B1636" s="0">
+        <v>19.738</v>
+      </c>
+      <c r="C1636" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1636" s="0">
+        <v>0.76458163652364897</v>
+      </c>
+    </row>
+    <row r="1637">
+      <c r="A1637" s="0">
+        <v>64.256110000000007</v>
+      </c>
+      <c r="B1637" s="0">
+        <v>19.7745</v>
+      </c>
+      <c r="C1637" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1637" s="0">
+        <v>0.79610475494392596</v>
+      </c>
+    </row>
+    <row r="1638">
+      <c r="A1638" s="0">
+        <v>-54.973300000000002</v>
+      </c>
+      <c r="B1638" s="0">
+        <v>-66.733500000000007</v>
+      </c>
+      <c r="C1638" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1638" s="0">
+        <v>0.78017168470128695</v>
+      </c>
+    </row>
+    <row r="1639">
+      <c r="A1639" s="0">
+        <v>-16.498000000000001</v>
+      </c>
+      <c r="B1639" s="0">
+        <v>-56.411999999999999</v>
+      </c>
+      <c r="C1639" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1639" s="0">
+        <v>0.492423658891737</v>
+      </c>
+    </row>
+    <row r="1640">
+      <c r="A1640" s="0">
+        <v>52.695</v>
+      </c>
+      <c r="B1640" s="0">
+        <v>-83.9452</v>
+      </c>
+      <c r="C1640" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1640" s="0">
+        <v>0.74975589108487795</v>
+      </c>
+    </row>
+    <row r="1641">
+      <c r="A1641" s="0">
+        <v>52.700800000000001</v>
+      </c>
+      <c r="B1641" s="0">
+        <v>-83.954999999999998</v>
+      </c>
+      <c r="C1641" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1641" s="0">
+        <v>0.76426638657697399</v>
+      </c>
+    </row>
+    <row r="1642">
+      <c r="A1642" s="0">
+        <v>49.8673</v>
+      </c>
+      <c r="B1642" s="0">
+        <v>-125.3336</v>
+      </c>
+      <c r="C1642" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1642" s="0">
+        <v>0.60451375547412001</v>
+      </c>
+    </row>
+    <row r="1643">
+      <c r="A1643" s="0">
+        <v>49.8705</v>
+      </c>
+      <c r="B1643" s="0">
+        <v>-125.29089999999999</v>
+      </c>
+      <c r="C1643" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1643" s="0">
+        <v>0.74668005621663203</v>
+      </c>
+    </row>
+    <row r="1644">
+      <c r="A1644" s="0">
+        <v>44.316699999999997</v>
+      </c>
+      <c r="B1644" s="0">
+        <v>-79.933300000000003</v>
+      </c>
+      <c r="C1644" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1644" s="0">
+        <v>0.88056119803307498</v>
+      </c>
+    </row>
+    <row r="1645">
+      <c r="A1645" s="0">
+        <v>49.129300000000001</v>
+      </c>
+      <c r="B1645" s="0">
+        <v>-122.9849</v>
+      </c>
+      <c r="C1645" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1645" s="0">
+        <v>0.857256645834367</v>
+      </c>
+    </row>
+    <row r="1646">
+      <c r="A1646" s="0">
+        <v>48.216700000000003</v>
+      </c>
+      <c r="B1646" s="0">
+        <v>-82.155600000000007</v>
+      </c>
+      <c r="C1646" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1646" s="0">
+        <v>0.84530058806681596</v>
+      </c>
+    </row>
+    <row r="1647">
+      <c r="A1647" s="0">
+        <v>55.111899999999999</v>
+      </c>
+      <c r="B1647" s="0">
+        <v>-122.84139999999999</v>
+      </c>
+      <c r="C1647" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1647" s="0">
+        <v>0.79603314585438201</v>
+      </c>
+    </row>
+    <row r="1648">
+      <c r="A1648" s="0">
+        <v>50.170999999999999</v>
+      </c>
+      <c r="B1648" s="0">
+        <v>-97.876199999999997</v>
+      </c>
+      <c r="C1648" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1648" s="0">
+        <v>0.81663638495481705</v>
+      </c>
+    </row>
+    <row r="1649">
+      <c r="A1649" s="0">
+        <v>50.177399999999999</v>
+      </c>
+      <c r="B1649" s="0">
+        <v>-97.868600000000001</v>
+      </c>
+      <c r="C1649" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1649" s="0">
+        <v>0.81829360332595302</v>
+      </c>
+    </row>
+    <row r="1650">
+      <c r="A1650" s="0">
+        <v>55.879199999999997</v>
+      </c>
+      <c r="B1650" s="0">
+        <v>-98.483900000000006</v>
+      </c>
+      <c r="C1650" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1650" s="0">
+        <v>0.75775478612099001</v>
+      </c>
+    </row>
+    <row r="1651">
+      <c r="A1651" s="0">
+        <v>55.905799999999999</v>
+      </c>
+      <c r="B1651" s="0">
+        <v>-98.524699999999996</v>
+      </c>
+      <c r="C1651" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1651" s="0">
+        <v>0.83282875815915403</v>
+      </c>
+    </row>
+    <row r="1652">
+      <c r="A1652" s="0">
+        <v>55.911700000000003</v>
+      </c>
+      <c r="B1652" s="0">
+        <v>-98.382199999999998</v>
+      </c>
+      <c r="C1652" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1652" s="0">
+        <v>0.74732986163686799</v>
+      </c>
+    </row>
+    <row r="1653">
+      <c r="A1653" s="0">
+        <v>55.914400000000001</v>
+      </c>
+      <c r="B1653" s="0">
+        <v>-98.380600000000001</v>
+      </c>
+      <c r="C1653" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1653" s="0">
+        <v>0.75536119960112902</v>
+      </c>
+    </row>
+    <row r="1654">
+      <c r="A1654" s="0">
+        <v>55.863100000000003</v>
+      </c>
+      <c r="B1654" s="0">
+        <v>-98.485</v>
+      </c>
+      <c r="C1654" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1654" s="0">
+        <v>0.83476024155039996</v>
+      </c>
+    </row>
+    <row r="1655">
+      <c r="A1655" s="0">
+        <v>55.916699999999999</v>
+      </c>
+      <c r="B1655" s="0">
+        <v>-98.964399999999998</v>
+      </c>
+      <c r="C1655" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1655" s="0">
+        <v>0.75580804662150503</v>
+      </c>
+    </row>
+    <row r="1656">
+      <c r="A1656" s="0">
+        <v>56.635800000000003</v>
+      </c>
+      <c r="B1656" s="0">
+        <v>-99.948300000000003</v>
+      </c>
+      <c r="C1656" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1656" s="0">
+        <v>0.76058434947244202</v>
+      </c>
+    </row>
+    <row r="1657">
+      <c r="A1657" s="0">
+        <v>49.692500000000003</v>
+      </c>
+      <c r="B1657" s="0">
+        <v>-74.342100000000002</v>
+      </c>
+      <c r="C1657" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1657" s="0">
+        <v>0.82274814889380599</v>
+      </c>
+    </row>
+    <row r="1658">
+      <c r="A1658" s="0">
+        <v>54.485</v>
+      </c>
+      <c r="B1658" s="0">
+        <v>-105.8176</v>
+      </c>
+      <c r="C1658" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1658" s="0">
+        <v>0.774845419743174</v>
+      </c>
+    </row>
+    <row r="1659">
+      <c r="A1659" s="0">
+        <v>54.253900000000002</v>
+      </c>
+      <c r="B1659" s="0">
+        <v>-105.8775</v>
+      </c>
+      <c r="C1659" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1659" s="0">
+        <v>0.80089245403231602</v>
+      </c>
+    </row>
+    <row r="1660">
+      <c r="A1660" s="0">
+        <v>42.660899999999998</v>
+      </c>
+      <c r="B1660" s="0">
+        <v>-80.5595</v>
+      </c>
+      <c r="C1660" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1660" s="0">
+        <v>0.765129468691232</v>
+      </c>
+    </row>
+    <row r="1661">
+      <c r="A1661" s="0">
+        <v>42.706800000000001</v>
+      </c>
+      <c r="B1661" s="0">
+        <v>-80.348299999999995</v>
+      </c>
+      <c r="C1661" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1661" s="0">
+        <v>0.84274434553538602</v>
+      </c>
+    </row>
+    <row r="1662">
+      <c r="A1662" s="0">
+        <v>42.635300000000001</v>
+      </c>
+      <c r="B1662" s="0">
+        <v>-80.557699999999997</v>
+      </c>
+      <c r="C1662" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1662" s="0">
+        <v>0.815697889289833</v>
+      </c>
+    </row>
+    <row r="1663">
+      <c r="A1663" s="0">
+        <v>27.84</v>
+      </c>
+      <c r="B1663" s="0">
+        <v>-109.3</v>
+      </c>
+      <c r="C1663" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1663" s="0">
+        <v>0.75595376607038101</v>
+      </c>
+    </row>
+    <row r="1664">
+      <c r="A1664" s="0">
+        <v>36.819299999999998</v>
+      </c>
+      <c r="B1664" s="0">
+        <v>-97.819800000000001</v>
+      </c>
+      <c r="C1664" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1664" s="0">
+        <v>0.088525984754249706</v>
+      </c>
+    </row>
+    <row r="1665">
+      <c r="A1665" s="0">
+        <v>46.030799999999999</v>
+      </c>
+      <c r="B1665" s="0">
+        <v>-89.606700000000004</v>
+      </c>
+      <c r="C1665" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1665" s="0">
+        <v>0.80906016218348198</v>
+      </c>
+    </row>
+    <row r="1666">
+      <c r="A1666" s="0">
+        <v>36.426699999999997</v>
+      </c>
+      <c r="B1666" s="0">
+        <v>-99.420000000000002</v>
+      </c>
+      <c r="C1666" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1666" s="0">
+        <v>0.65880677454083403</v>
+      </c>
+    </row>
+    <row r="1667">
+      <c r="A1667" s="0">
+        <v>36.635800000000003</v>
+      </c>
+      <c r="B1667" s="0">
+        <v>-99.597499999999997</v>
+      </c>
+      <c r="C1667" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1667" s="0">
+        <v>0.62796992541854002</v>
+      </c>
+    </row>
+    <row r="1668">
+      <c r="A1668" s="0">
+        <v>39.216700000000003</v>
+      </c>
+      <c r="B1668" s="0">
+        <v>-86.540599999999998</v>
+      </c>
+      <c r="C1668" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1668" s="0">
+        <v>0.89083197740726805</v>
+      </c>
+    </row>
+    <row r="1669">
+      <c r="A1669" s="0">
+        <v>64.695499999999996</v>
+      </c>
+      <c r="B1669" s="0">
+        <v>-148.32079999999999</v>
+      </c>
+      <c r="C1669" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1669" s="0">
+        <v>0.77036737631830299</v>
+      </c>
+    </row>
+    <row r="1670">
+      <c r="A1670" s="0">
+        <v>64.701300000000003</v>
+      </c>
+      <c r="B1670" s="0">
+        <v>-148.31209999999999</v>
+      </c>
+      <c r="C1670" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1670" s="0">
+        <v>0.80646185728429698</v>
+      </c>
+    </row>
+    <row r="1671">
+      <c r="A1671" s="0">
+        <v>64.696299999999994</v>
+      </c>
+      <c r="B1671" s="0">
+        <v>-148.3235</v>
+      </c>
+      <c r="C1671" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1671" s="0">
+        <v>0.75938900134695597</v>
+      </c>
+    </row>
+    <row r="1672">
+      <c r="A1672" s="0">
+        <v>64.693600000000004</v>
+      </c>
+      <c r="B1672" s="0">
+        <v>-148.33000000000001</v>
+      </c>
+      <c r="C1672" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1672" s="0">
+        <v>0.86947826883535395</v>
+      </c>
+    </row>
+    <row r="1673">
+      <c r="A1673" s="0">
+        <v>44.064599999999999</v>
+      </c>
+      <c r="B1673" s="0">
+        <v>-71.2881</v>
+      </c>
+      <c r="C1673" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1673" s="0">
+        <v>0.87404935724823596</v>
+      </c>
+    </row>
+    <row r="1674">
+      <c r="A1674" s="0">
+        <v>44.146700000000003</v>
+      </c>
+      <c r="B1674" s="0">
+        <v>-89.500200000000007</v>
+      </c>
+      <c r="C1674" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1674" s="0">
+        <v>0.85670203977923298</v>
+      </c>
+    </row>
+    <row r="1675">
+      <c r="A1675" s="0">
+        <v>63.878399999999999</v>
+      </c>
+      <c r="B1675" s="0">
+        <v>-149.25360000000001</v>
+      </c>
+      <c r="C1675" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1675" s="0">
+        <v>0.77556663470110998</v>
+      </c>
+    </row>
+    <row r="1676">
+      <c r="A1676" s="0">
+        <v>65.396799999999999</v>
+      </c>
+      <c r="B1676" s="0">
+        <v>-148.9348</v>
+      </c>
+      <c r="C1676" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1676" s="0">
+        <v>0.81612392726578698</v>
+      </c>
+    </row>
+    <row r="1677">
+      <c r="A1677" s="0">
+        <v>35.142600000000002</v>
+      </c>
+      <c r="B1677" s="0">
+        <v>-111.7273</v>
+      </c>
+      <c r="C1677" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1677" s="0">
+        <v>0.37663680659490201</v>
+      </c>
+    </row>
+    <row r="1678">
+      <c r="A1678" s="0">
+        <v>35.088999999999999</v>
+      </c>
+      <c r="B1678" s="0">
+        <v>-111.762</v>
+      </c>
+      <c r="C1678" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1678" s="0">
+        <v>0.78026936216817</v>
+      </c>
+    </row>
+    <row r="1679">
+      <c r="A1679" s="0">
+        <v>41.366500000000002</v>
+      </c>
+      <c r="B1679" s="0">
+        <v>-106.23990000000001</v>
+      </c>
+      <c r="C1679" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1679" s="0">
+        <v>0.77078243476850095</v>
+      </c>
+    </row>
+    <row r="1680">
+      <c r="A1680" s="0">
+        <v>42.537799999999997</v>
+      </c>
+      <c r="B1680" s="0">
+        <v>-72.171499999999995</v>
+      </c>
+      <c r="C1680" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1680" s="0">
+        <v>0.82989668303177999</v>
+      </c>
+    </row>
+    <row r="1681">
+      <c r="A1681" s="0">
+        <v>45.209099999999999</v>
+      </c>
+      <c r="B1681" s="0">
+        <v>-68.747</v>
+      </c>
+      <c r="C1681" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1681" s="0">
+        <v>0.74752995427461599</v>
+      </c>
+    </row>
+    <row r="1682">
+      <c r="A1682" s="0">
+        <v>68.606800000000007</v>
+      </c>
+      <c r="B1682" s="0">
+        <v>-149.29580000000001</v>
+      </c>
+      <c r="C1682" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1682" s="0">
+        <v>0.57884904207148003</v>
+      </c>
+    </row>
+    <row r="1683">
+      <c r="A1683" s="0">
+        <v>68.605800000000002</v>
+      </c>
+      <c r="B1683" s="0">
+        <v>-149.31100000000001</v>
+      </c>
+      <c r="C1683" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1683" s="0">
+        <v>0.55025880369125402</v>
+      </c>
+    </row>
+    <row r="1684">
+      <c r="A1684" s="0">
+        <v>68.606300000000005</v>
+      </c>
+      <c r="B1684" s="0">
+        <v>-149.30410000000001</v>
+      </c>
+      <c r="C1684" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1684" s="0">
+        <v>0.55706297444423703</v>
+      </c>
+    </row>
+    <row r="1685">
+      <c r="A1685" s="0">
+        <v>32.582000000000001</v>
+      </c>
+      <c r="B1685" s="0">
+        <v>-106.63500000000001</v>
+      </c>
+      <c r="C1685" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1685" s="0">
+        <v>0.430309108768061</v>
+      </c>
+    </row>
+    <row r="1686">
+      <c r="A1686" s="0">
+        <v>32.584899999999998</v>
+      </c>
+      <c r="B1686" s="0">
+        <v>-106.6032</v>
+      </c>
+      <c r="C1686" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1686" s="0">
+        <v>0.45970034556438699</v>
+      </c>
+    </row>
+    <row r="1687">
+      <c r="A1687" s="0">
+        <v>39.056100000000001</v>
+      </c>
+      <c r="B1687" s="0">
+        <v>-95.190700000000007</v>
+      </c>
+      <c r="C1687" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1687" s="0">
+        <v>0.75397983235087196</v>
+      </c>
+    </row>
+    <row r="1688">
+      <c r="A1688" s="0">
+        <v>38.774500000000003</v>
+      </c>
+      <c r="B1688" s="0">
+        <v>-97.568399999999997</v>
+      </c>
+      <c r="C1688" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1688" s="0">
+        <v>0.66798448721530901</v>
+      </c>
+    </row>
+    <row r="1689">
+      <c r="A1689" s="0">
+        <v>31.565899999999999</v>
+      </c>
+      <c r="B1689" s="0">
+        <v>-110.1344</v>
+      </c>
+      <c r="C1689" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1689" s="0">
+        <v>0.67783357182024195</v>
+      </c>
+    </row>
+    <row r="1690">
+      <c r="A1690" s="0">
+        <v>39.3232</v>
+      </c>
+      <c r="B1690" s="0">
+        <v>-86.4131</v>
+      </c>
+      <c r="C1690" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1690" s="0">
+        <v>0.82489580687331698</v>
+      </c>
+    </row>
+    <row r="1691">
+      <c r="A1691" s="0">
+        <v>38.744100000000003</v>
+      </c>
+      <c r="B1691" s="0">
+        <v>-92.200000000000003</v>
+      </c>
+      <c r="C1691" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1691" s="0">
+        <v>0.76536336974111896</v>
+      </c>
+    </row>
+    <row r="1692">
+      <c r="A1692" s="0">
+        <v>44.452300000000001</v>
+      </c>
+      <c r="B1692" s="0">
+        <v>-121.5574</v>
+      </c>
+      <c r="C1692" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1692" s="0">
+        <v>0.27899121809041399</v>
+      </c>
+    </row>
+    <row r="1693">
+      <c r="A1693" s="0">
+        <v>44.315399999999997</v>
+      </c>
+      <c r="B1693" s="0">
+        <v>-121.6078</v>
+      </c>
+      <c r="C1693" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1693" s="0">
+        <v>0.28390734585702099</v>
+      </c>
+    </row>
+    <row r="1694">
+      <c r="A1694" s="0">
+        <v>34.438499999999998</v>
+      </c>
+      <c r="B1694" s="0">
+        <v>-106.2377</v>
+      </c>
+      <c r="C1694" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1694" s="0">
+        <v>0.80245730645832802</v>
+      </c>
+    </row>
+    <row r="1695">
+      <c r="A1695" s="0">
+        <v>38.049900000000001</v>
+      </c>
+      <c r="B1695" s="0">
+        <v>-121.765</v>
+      </c>
+      <c r="C1695" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1695" s="0">
+        <v>0.64303582828434502</v>
+      </c>
+    </row>
+    <row r="1696">
+      <c r="A1696" s="0">
+        <v>35.811799999999998</v>
+      </c>
+      <c r="B1696" s="0">
+        <v>-76.7119</v>
+      </c>
+      <c r="C1696" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1696" s="0">
+        <v>0.70112616449834697</v>
+      </c>
+    </row>
+    <row r="1697">
+      <c r="A1697" s="0">
+        <v>35.799</v>
+      </c>
+      <c r="B1697" s="0">
+        <v>-76.656000000000006</v>
+      </c>
+      <c r="C1697" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1697" s="0">
+        <v>0.45472061410982501</v>
+      </c>
+    </row>
+    <row r="1698">
+      <c r="A1698" s="0">
+        <v>35.7879</v>
+      </c>
+      <c r="B1698" s="0">
+        <v>-75.903800000000004</v>
+      </c>
+      <c r="C1698" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1698" s="0">
+        <v>0.63635368304344397</v>
+      </c>
+    </row>
+    <row r="1699">
+      <c r="A1699" s="0">
+        <v>64.861400000000003</v>
+      </c>
+      <c r="B1699" s="0">
+        <v>-163.70079999999999</v>
+      </c>
+      <c r="C1699" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1699" s="0">
+        <v>0.59834206269083201</v>
+      </c>
+    </row>
+    <row r="1700">
+      <c r="A1700" s="0">
+        <v>40.032899999999998</v>
+      </c>
+      <c r="B1700" s="0">
+        <v>-105.54640000000001</v>
+      </c>
+      <c r="C1700" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1700" s="0">
+        <v>0.82485325180814195</v>
+      </c>
+    </row>
+    <row r="1701">
+      <c r="A1701" s="0">
+        <v>27.383600000000001</v>
+      </c>
+      <c r="B1701" s="0">
+        <v>-81.950900000000004</v>
+      </c>
+      <c r="C1701" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1701" s="0">
+        <v>0.49121732948776098</v>
+      </c>
+    </row>
+    <row r="1702">
+      <c r="A1702" s="0">
+        <v>40.020099999999999</v>
+      </c>
+      <c r="B1702" s="0">
+        <v>-83.018299999999997</v>
+      </c>
+      <c r="C1702" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1702" s="0"/>
+    </row>
+    <row r="1703">
+      <c r="A1703" s="0">
+        <v>43.064500000000002</v>
+      </c>
+      <c r="B1703" s="0">
+        <v>-116.7486</v>
+      </c>
+      <c r="C1703" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1703" s="0">
+        <v>0.84460512023163004</v>
+      </c>
+    </row>
+    <row r="1704">
+      <c r="A1704" s="0">
+        <v>44.678100000000001</v>
+      </c>
+      <c r="B1704" s="0">
+        <v>-93.072299999999999</v>
+      </c>
+      <c r="C1704" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1704" s="0">
+        <v>0.84820446370453395</v>
+      </c>
+    </row>
+    <row r="1705">
+      <c r="A1705" s="0">
+        <v>43.065300000000001</v>
+      </c>
+      <c r="B1705" s="0">
+        <v>-116.7591</v>
+      </c>
+      <c r="C1705" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1705" s="0">
+        <v>0.75272745155023402</v>
+      </c>
+    </row>
+    <row r="1706">
+      <c r="A1706" s="0">
+        <v>43.120699999999999</v>
+      </c>
+      <c r="B1706" s="0">
+        <v>-116.7231</v>
+      </c>
+      <c r="C1706" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1706" s="0">
+        <v>0.84065409174837003</v>
+      </c>
+    </row>
+    <row r="1707">
+      <c r="A1707" s="0">
+        <v>43.167499999999997</v>
+      </c>
+      <c r="B1707" s="0">
+        <v>-116.7132</v>
+      </c>
+      <c r="C1707" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1707" s="0">
+        <v>0.742948506500547</v>
+      </c>
+    </row>
+    <row r="1708">
+      <c r="A1708" s="0">
+        <v>31.908300000000001</v>
+      </c>
+      <c r="B1708" s="0">
+        <v>-110.8395</v>
+      </c>
+      <c r="C1708" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1708" s="0">
+        <v>0.51583127936348006</v>
+      </c>
+    </row>
+    <row r="1709">
+      <c r="A1709" s="0">
+        <v>31.789400000000001</v>
+      </c>
+      <c r="B1709" s="0">
+        <v>-110.82769999999999</v>
+      </c>
+      <c r="C1709" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1709" s="0">
+        <v>0.58168740096064098</v>
+      </c>
+    </row>
+    <row r="1710">
+      <c r="A1710" s="0">
+        <v>31.8173</v>
+      </c>
+      <c r="B1710" s="0">
+        <v>-110.85080000000001</v>
+      </c>
+      <c r="C1710" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1710" s="0">
+        <v>0.41423776210501101</v>
+      </c>
+    </row>
+    <row r="1711">
+      <c r="A1711" s="0">
+        <v>34.362299999999998</v>
+      </c>
+      <c r="B1711" s="0">
+        <v>-106.702</v>
+      </c>
+      <c r="C1711" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1711" s="0">
+        <v>0.60012117502693396</v>
+      </c>
+    </row>
+    <row r="1712">
+      <c r="A1712" s="0">
+        <v>34.334899999999998</v>
+      </c>
+      <c r="B1712" s="0">
+        <v>-106.74420000000001</v>
+      </c>
+      <c r="C1712" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1712" s="0">
+        <v>0.61796671113157098</v>
+      </c>
+    </row>
+    <row r="1713">
+      <c r="A1713" s="0">
+        <v>38.036900000000003</v>
+      </c>
+      <c r="B1713" s="0">
+        <v>-121.7547</v>
+      </c>
+      <c r="C1713" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1713" s="0">
+        <v>0.58024472901090796</v>
+      </c>
+    </row>
+    <row r="1714">
+      <c r="A1714" s="0">
+        <v>38.040199999999999</v>
+      </c>
+      <c r="B1714" s="0">
+        <v>-121.7272</v>
+      </c>
+      <c r="C1714" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1714" s="0">
+        <v>0.74310048464475598</v>
+      </c>
+    </row>
+    <row r="1715">
+      <c r="A1715" s="0">
+        <v>46.241999999999997</v>
+      </c>
+      <c r="B1715" s="0">
+        <v>-89.347700000000003</v>
+      </c>
+      <c r="C1715" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1715" s="0">
+        <v>0.86195958383150995</v>
+      </c>
+    </row>
+    <row r="1716">
+      <c r="A1716" s="0">
+        <v>38.430900000000001</v>
+      </c>
+      <c r="B1716" s="0">
+        <v>-120.96599999999999</v>
+      </c>
+      <c r="C1716" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1716" s="0">
+        <v>0.64193047585903396</v>
+      </c>
+    </row>
+    <row r="1717">
+      <c r="A1717" s="0">
+        <v>38.107399999999998</v>
+      </c>
+      <c r="B1717" s="0">
+        <v>-121.6469</v>
+      </c>
+      <c r="C1717" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1717" s="0">
+        <v>0.32548447645152401</v>
+      </c>
+    </row>
+    <row r="1718">
+      <c r="A1718" s="0">
+        <v>38.102699999999999</v>
+      </c>
+      <c r="B1718" s="0">
+        <v>-121.6413</v>
+      </c>
+      <c r="C1718" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1718" s="0">
+        <v>0.211464258145623</v>
+      </c>
+    </row>
+    <row r="1719">
+      <c r="A1719" s="0">
+        <v>45.559800000000003</v>
+      </c>
+      <c r="B1719" s="0">
+        <v>-84.713800000000006</v>
+      </c>
+      <c r="C1719" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1719" s="0">
+        <v>0.80713653109884498</v>
+      </c>
+    </row>
+    <row r="1720">
+      <c r="A1720" s="0">
+        <v>45.5625</v>
+      </c>
+      <c r="B1720" s="0">
+        <v>-84.697500000000005</v>
+      </c>
+      <c r="C1720" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1720" s="0">
+        <v>0.82036020782150298</v>
+      </c>
+    </row>
+    <row r="1721">
+      <c r="A1721" s="0">
+        <v>38.4133</v>
+      </c>
+      <c r="B1721" s="0">
+        <v>-120.9508</v>
+      </c>
+      <c r="C1721" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1721" s="0">
+        <v>0.63394010788878596</v>
+      </c>
+    </row>
+    <row r="1722">
+      <c r="A1722" s="0">
+        <v>31.7438</v>
+      </c>
+      <c r="B1722" s="0">
+        <v>-110.0522</v>
+      </c>
+      <c r="C1722" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1722" s="0">
+        <v>0.63452410715013696</v>
+      </c>
+    </row>
+    <row r="1723">
+      <c r="A1723" s="0">
+        <v>34.4255</v>
+      </c>
+      <c r="B1723" s="0">
+        <v>-105.86150000000001</v>
+      </c>
+      <c r="C1723" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1723" s="0">
+        <v>0.74074006419402005</v>
+      </c>
+    </row>
+    <row r="1724">
+      <c r="A1724" s="0">
+        <v>31.7365</v>
+      </c>
+      <c r="B1724" s="0">
+        <v>-109.9419</v>
+      </c>
+      <c r="C1724" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1724" s="0">
+        <v>0.66964785977202501</v>
+      </c>
+    </row>
+    <row r="1725">
+      <c r="A1725" s="0">
+        <v>35.410600000000002</v>
+      </c>
+      <c r="B1725" s="0">
+        <v>-99.058800000000005</v>
+      </c>
+      <c r="C1725" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1725" s="0">
+        <v>0.66931961505514204</v>
+      </c>
+    </row>
+    <row r="1726">
+      <c r="A1726" s="0">
+        <v>44.063899999999997</v>
+      </c>
+      <c r="B1726" s="0">
+        <v>-71.287300000000002</v>
+      </c>
+      <c r="C1726" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1726" s="0">
+        <v>0.88288327709852099</v>
+      </c>
+    </row>
+    <row r="1727">
+      <c r="A1727" s="0">
+        <v>33.401200000000003</v>
+      </c>
+      <c r="B1727" s="0">
+        <v>-97.569999999999993</v>
+      </c>
+      <c r="C1727" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1727" s="0">
+        <v>0.40177566460393599</v>
+      </c>
+    </row>
+    <row r="1728">
+      <c r="A1728" s="0">
+        <v>40.8155</v>
+      </c>
+      <c r="B1728" s="0">
+        <v>-104.7456</v>
+      </c>
+      <c r="C1728" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1728" s="0">
+        <v>0.82945911778661996</v>
+      </c>
+    </row>
+    <row r="1729">
+      <c r="A1729" s="0">
+        <v>47.161700000000003</v>
+      </c>
+      <c r="B1729" s="0">
+        <v>-99.1066</v>
+      </c>
+      <c r="C1729" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1729" s="0">
+        <v>0.86673074128910899</v>
+      </c>
+    </row>
+    <row r="1730">
+      <c r="A1730" s="0">
+        <v>32.541699999999999</v>
+      </c>
+      <c r="B1730" s="0">
+        <v>-87.803899999999999</v>
+      </c>
+      <c r="C1730" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1730" s="0">
+        <v>0.70696055473963604</v>
+      </c>
+    </row>
+    <row r="1731">
+      <c r="A1731" s="0">
+        <v>35.689</v>
+      </c>
+      <c r="B1731" s="0">
+        <v>-83.501900000000006</v>
+      </c>
+      <c r="C1731" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1731" s="0">
+        <v>0.79365869778267495</v>
+      </c>
+    </row>
+    <row r="1732">
+      <c r="A1732" s="0">
+        <v>42.536900000000003</v>
+      </c>
+      <c r="B1732" s="0">
+        <v>-72.172700000000006</v>
+      </c>
+      <c r="C1732" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1732" s="0">
+        <v>0.86333505669154698</v>
+      </c>
+    </row>
+    <row r="1733">
+      <c r="A1733" s="0">
+        <v>63.875700000000002</v>
+      </c>
+      <c r="B1733" s="0">
+        <v>-149.2133</v>
+      </c>
+      <c r="C1733" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1733" s="0">
+        <v>0.70232635850543102</v>
+      </c>
+    </row>
+    <row r="1734">
+      <c r="A1734" s="0">
+        <v>31.194800000000001</v>
+      </c>
+      <c r="B1734" s="0">
+        <v>-84.468599999999995</v>
+      </c>
+      <c r="C1734" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1734" s="0">
+        <v>0.52876519563120306</v>
+      </c>
+    </row>
+    <row r="1735">
+      <c r="A1735" s="0">
+        <v>39.110399999999999</v>
+      </c>
+      <c r="B1735" s="0">
+        <v>-96.612899999999996</v>
+      </c>
+      <c r="C1735" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1735" s="0">
+        <v>0.50649688541237803</v>
+      </c>
+    </row>
+    <row r="1736">
+      <c r="A1736" s="0">
+        <v>39.1008</v>
+      </c>
+      <c r="B1736" s="0">
+        <v>-96.563100000000006</v>
+      </c>
+      <c r="C1736" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1736" s="0">
+        <v>0.71817059858117804</v>
+      </c>
+    </row>
+    <row r="1737">
+      <c r="A1737" s="0">
+        <v>38.2483</v>
+      </c>
+      <c r="B1737" s="0">
+        <v>-109.3883</v>
+      </c>
+      <c r="C1737" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1737" s="0">
+        <v>0.67999488961169596</v>
+      </c>
+    </row>
+    <row r="1738">
+      <c r="A1738" s="0">
+        <v>37.378300000000003</v>
+      </c>
+      <c r="B1738" s="0">
+        <v>-80.524799999999999</v>
+      </c>
+      <c r="C1738" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1738" s="0">
+        <v>0.81225363743213697</v>
+      </c>
+    </row>
+    <row r="1739">
+      <c r="A1739" s="0">
+        <v>46.7697</v>
+      </c>
+      <c r="B1739" s="0">
+        <v>-100.91540000000001</v>
+      </c>
+      <c r="C1739" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1739" s="0">
+        <v>0.78081940897211599</v>
+      </c>
+    </row>
+    <row r="1740">
+      <c r="A1740" s="0">
+        <v>40.177599999999998</v>
+      </c>
+      <c r="B1740" s="0">
+        <v>-112.4524</v>
+      </c>
+      <c r="C1740" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1740" s="0">
+        <v>0.66067974272045205</v>
+      </c>
+    </row>
+    <row r="1741">
+      <c r="A1741" s="0">
+        <v>40.2759</v>
+      </c>
+      <c r="B1741" s="0">
+        <v>-105.5459</v>
+      </c>
+      <c r="C1741" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1741" s="0">
+        <v>0.63621432598597305</v>
+      </c>
+    </row>
+    <row r="1742">
+      <c r="A1742" s="0">
+        <v>29.689299999999999</v>
+      </c>
+      <c r="B1742" s="0">
+        <v>-81.993399999999994</v>
+      </c>
+      <c r="C1742" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1742" s="0">
+        <v>0.55642056641300297</v>
+      </c>
+    </row>
+    <row r="1743">
+      <c r="A1743" s="0">
+        <v>38.890099999999997</v>
+      </c>
+      <c r="B1743" s="0">
+        <v>-76.560000000000002</v>
+      </c>
+      <c r="C1743" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1743" s="0">
+        <v>0.79751271643836896</v>
+      </c>
+    </row>
+    <row r="1744">
+      <c r="A1744" s="0">
+        <v>31.910699999999999</v>
+      </c>
+      <c r="B1744" s="0">
+        <v>-110.8355</v>
+      </c>
+      <c r="C1744" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1744" s="0">
+        <v>0.44032820845985499</v>
+      </c>
+    </row>
+    <row r="1745">
+      <c r="A1745" s="0">
+        <v>45.508899999999997</v>
+      </c>
+      <c r="B1745" s="0">
+        <v>-89.586399999999998</v>
+      </c>
+      <c r="C1745" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1745" s="0">
+        <v>0.88487750688460698</v>
+      </c>
+    </row>
+    <row r="1746">
+      <c r="A1746" s="0">
+        <v>32.950499999999998</v>
+      </c>
+      <c r="B1746" s="0">
+        <v>-87.393299999999997</v>
+      </c>
+      <c r="C1746" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1746" s="0">
+        <v>0.71863256736425396</v>
+      </c>
+    </row>
+    <row r="1747">
+      <c r="A1747" s="0">
+        <v>45.493699999999997</v>
+      </c>
+      <c r="B1747" s="0">
+        <v>-89.585700000000003</v>
+      </c>
+      <c r="C1747" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1747" s="0">
+        <v>0.88989856728374495</v>
+      </c>
+    </row>
+    <row r="1748">
+      <c r="A1748" s="0">
+        <v>39.040399999999998</v>
+      </c>
+      <c r="B1748" s="0">
+        <v>-95.192099999999996</v>
+      </c>
+      <c r="C1748" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1748" s="0">
+        <v>0.79548206932256405</v>
+      </c>
+    </row>
+    <row r="1749">
+      <c r="A1749" s="0">
+        <v>46.233899999999999</v>
+      </c>
+      <c r="B1749" s="0">
+        <v>-89.537300000000002</v>
+      </c>
+      <c r="C1749" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1749" s="0">
+        <v>0.86140923996424601</v>
+      </c>
+    </row>
+    <row r="1750">
+      <c r="A1750" s="0">
+        <v>44.953499999999998</v>
+      </c>
+      <c r="B1750" s="0">
+        <v>-110.5391</v>
+      </c>
+      <c r="C1750" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1750" s="0">
+        <v>0.88382338292889096</v>
+      </c>
+    </row>
+    <row r="1751">
+      <c r="A1751" s="0">
+        <v>-33.464799999999997</v>
+      </c>
+      <c r="B1751" s="0">
+        <v>-66.459800000000001</v>
+      </c>
+      <c r="C1751" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1751" s="0">
+        <v>0.827680211179597</v>
+      </c>
+    </row>
+    <row r="1752">
+      <c r="A1752" s="0">
+        <v>47.116700000000002</v>
+      </c>
+      <c r="B1752" s="0">
+        <v>11.317500000000001</v>
+      </c>
+      <c r="C1752" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1752" s="0">
+        <v>0.79573626827489197</v>
+      </c>
+    </row>
+    <row r="1753">
+      <c r="A1753" s="0">
+        <v>-22.283000000000001</v>
+      </c>
+      <c r="B1753" s="0">
+        <v>133.249</v>
+      </c>
+      <c r="C1753" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1753" s="0">
+        <v>0.56978454241114096</v>
+      </c>
+    </row>
+    <row r="1754">
+      <c r="A1754" s="0">
+        <v>-13.0769</v>
+      </c>
+      <c r="B1754" s="0">
+        <v>131.11779999999999</v>
+      </c>
+      <c r="C1754" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1754" s="0">
+        <v>0.74839314538185797</v>
+      </c>
+    </row>
+    <row r="1755">
+      <c r="A1755" s="0">
+        <v>-34.002099999999999</v>
+      </c>
+      <c r="B1755" s="0">
+        <v>140.5891</v>
+      </c>
+      <c r="C1755" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1755" s="0">
+        <v>0.017265858005232001</v>
+      </c>
+    </row>
+    <row r="1756">
+      <c r="A1756" s="0">
+        <v>-33.615200000000002</v>
+      </c>
+      <c r="B1756" s="0">
+        <v>150.7236</v>
+      </c>
+      <c r="C1756" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1756" s="0">
+        <v>0.52259730489720402</v>
+      </c>
+    </row>
+    <row r="1757">
+      <c r="A1757" s="0">
+        <v>-14.0633</v>
+      </c>
+      <c r="B1757" s="0">
+        <v>131.31809999999999</v>
+      </c>
+      <c r="C1757" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1757" s="0">
+        <v>0.79527499832606796</v>
+      </c>
+    </row>
+    <row r="1758">
+      <c r="A1758" s="0">
+        <v>-14.1593</v>
+      </c>
+      <c r="B1758" s="0">
+        <v>131.38810000000001</v>
+      </c>
+      <c r="C1758" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1758" s="0">
+        <v>0.73623636269153203</v>
+      </c>
+    </row>
+    <row r="1759">
+      <c r="A1759" s="0">
+        <v>-15.258800000000001</v>
+      </c>
+      <c r="B1759" s="0">
+        <v>132.3706</v>
+      </c>
+      <c r="C1759" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1759" s="0">
+        <v>0.72328611315525904</v>
+      </c>
+    </row>
+    <row r="1760">
+      <c r="A1760" s="0">
+        <v>-23.858699999999999</v>
+      </c>
+      <c r="B1760" s="0">
+        <v>148.47460000000001</v>
+      </c>
+      <c r="C1760" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1760" s="0">
+        <v>0.016207243717065799</v>
+      </c>
+    </row>
+    <row r="1761">
+      <c r="A1761" s="0">
+        <v>-12.545199999999999</v>
+      </c>
+      <c r="B1761" s="0">
+        <v>131.3072</v>
+      </c>
+      <c r="C1761" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1761" s="0">
+        <v>0.44480031287490901</v>
+      </c>
+    </row>
+    <row r="1762">
+      <c r="A1762" s="0">
+        <v>-31.3764</v>
+      </c>
+      <c r="B1762" s="0">
+        <v>115.71380000000001</v>
+      </c>
+      <c r="C1762" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1762" s="0">
+        <v>0.41661166684627998</v>
+      </c>
+    </row>
+    <row r="1763">
+      <c r="A1763" s="0">
+        <v>-12.494300000000001</v>
+      </c>
+      <c r="B1763" s="0">
+        <v>131.1523</v>
+      </c>
+      <c r="C1763" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1763" s="0">
+        <v>0.57283889232518104</v>
+      </c>
+    </row>
+    <row r="1764">
+      <c r="A1764" s="0">
+        <v>-14.563599999999999</v>
+      </c>
+      <c r="B1764" s="0">
+        <v>132.4776</v>
+      </c>
+      <c r="C1764" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1764" s="0">
+        <v>0.79391366973723199</v>
+      </c>
+    </row>
+    <row r="1765">
+      <c r="A1765" s="0">
+        <v>-36.649900000000002</v>
+      </c>
+      <c r="B1765" s="0">
+        <v>145.57589999999999</v>
+      </c>
+      <c r="C1765" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1765" s="0">
+        <v>-0.0507016732258617</v>
+      </c>
+    </row>
+    <row r="1766">
+      <c r="A1766" s="0">
+        <v>-17.150700000000001</v>
+      </c>
+      <c r="B1766" s="0">
+        <v>133.3502</v>
+      </c>
+      <c r="C1766" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1766" s="0">
+        <v>0.66110502367240598</v>
+      </c>
+    </row>
+    <row r="1767">
+      <c r="A1767" s="0">
+        <v>-22.286999999999999</v>
+      </c>
+      <c r="B1767" s="0">
+        <v>133.63999999999999</v>
+      </c>
+      <c r="C1767" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1767" s="0">
+        <v>0.27392673131898598</v>
+      </c>
+    </row>
+    <row r="1768">
+      <c r="A1768" s="0">
+        <v>-35.656599999999998</v>
+      </c>
+      <c r="B1768" s="0">
+        <v>148.15170000000001</v>
+      </c>
+      <c r="C1768" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1768" s="0">
+        <v>0.468988407528731</v>
+      </c>
+    </row>
+    <row r="1769">
+      <c r="A1769" s="0">
+        <v>-37.425899999999999</v>
+      </c>
+      <c r="B1769" s="0">
+        <v>145.18780000000001</v>
+      </c>
+      <c r="C1769" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1769" s="0">
+        <v>-0.16017578895223</v>
+      </c>
+    </row>
+    <row r="1770">
+      <c r="A1770" s="0">
+        <v>-37.422199999999997</v>
+      </c>
+      <c r="B1770" s="0">
+        <v>144.09440000000001</v>
+      </c>
+      <c r="C1770" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1770" s="0">
+        <v>0.072222418789341505</v>
+      </c>
+    </row>
+    <row r="1771">
+      <c r="A1771" s="0">
+        <v>-34.9893</v>
+      </c>
+      <c r="B1771" s="0">
+        <v>146.29069999999999</v>
+      </c>
+      <c r="C1771" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1771" s="0">
+        <v>-0.16632756652953501</v>
+      </c>
+    </row>
+    <row r="1772">
+      <c r="A1772" s="0">
+        <v>-3.0179999999999998</v>
+      </c>
+      <c r="B1772" s="0">
+        <v>-54.971400000000003</v>
+      </c>
+      <c r="C1772" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1772" s="0">
+        <v>0.11501000533408701</v>
+      </c>
+    </row>
+    <row r="1773">
+      <c r="A1773" s="0">
+        <v>55.879600000000004</v>
+      </c>
+      <c r="B1773" s="0">
+        <v>-98.480800000000002</v>
+      </c>
+      <c r="C1773" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1773" s="0">
+        <v>0.81097108057116596</v>
+      </c>
+    </row>
+    <row r="1774">
+      <c r="A1774" s="0">
+        <v>53.628900000000002</v>
+      </c>
+      <c r="B1774" s="0">
+        <v>-106.1978</v>
+      </c>
+      <c r="C1774" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1774" s="0">
+        <v>0.81678164906912998</v>
+      </c>
+    </row>
+    <row r="1775">
+      <c r="A1775" s="0">
+        <v>53.987200000000001</v>
+      </c>
+      <c r="B1775" s="0">
+        <v>-105.1178</v>
+      </c>
+      <c r="C1775" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1775" s="0">
+        <v>0.82874466380703205</v>
+      </c>
+    </row>
+    <row r="1776">
+      <c r="A1776" s="0">
+        <v>54.0916</v>
+      </c>
+      <c r="B1776" s="0">
+        <v>-106.00530000000001</v>
+      </c>
+      <c r="C1776" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1776" s="0">
+        <v>0.82231795189631296</v>
+      </c>
+    </row>
+    <row r="1777">
+      <c r="A1777" s="0">
+        <v>42.7744</v>
+      </c>
+      <c r="B1777" s="0">
+        <v>-80.458799999999997</v>
+      </c>
+      <c r="C1777" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1777" s="0">
+        <v>0.80414986036529901</v>
+      </c>
+    </row>
+    <row r="1778">
+      <c r="A1778" s="0">
+        <v>42.7102</v>
+      </c>
+      <c r="B1778" s="0">
+        <v>-80.357399999999998</v>
+      </c>
+      <c r="C1778" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1778" s="0">
+        <v>0.78266066540415802</v>
+      </c>
+    </row>
+    <row r="1779">
+      <c r="A1779" s="0">
+        <v>-4.2892000000000001</v>
+      </c>
+      <c r="B1779" s="0">
+        <v>11.6564</v>
+      </c>
+      <c r="C1779" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1779" s="0">
+        <v>0.62544484131917</v>
+      </c>
+    </row>
+    <row r="1780">
+      <c r="A1780" s="0">
+        <v>47.285800000000002</v>
+      </c>
+      <c r="B1780" s="0">
+        <v>7.7319000000000004</v>
+      </c>
+      <c r="C1780" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1780" s="0">
+        <v>0.79174211411792506</v>
+      </c>
+    </row>
+    <row r="1781">
+      <c r="A1781" s="0">
+        <v>42.402500000000004</v>
+      </c>
+      <c r="B1781" s="0">
+        <v>128.0958</v>
+      </c>
+      <c r="C1781" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1781" s="0">
+        <v>0.86778210504114495</v>
+      </c>
+    </row>
+    <row r="1782">
+      <c r="A1782" s="0">
+        <v>44.593400000000003</v>
+      </c>
+      <c r="B1782" s="0">
+        <v>123.50920000000001</v>
+      </c>
+      <c r="C1782" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1782" s="0">
+        <v>0.75286600199700804</v>
+      </c>
+    </row>
+    <row r="1783">
+      <c r="A1783" s="0">
+        <v>23.173300000000001</v>
+      </c>
+      <c r="B1783" s="0">
+        <v>112.5361</v>
+      </c>
+      <c r="C1783" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1783" s="0">
+        <v>0.28182835532414302</v>
+      </c>
+    </row>
+    <row r="1784">
+      <c r="A1784" s="0">
+        <v>42.046700000000001</v>
+      </c>
+      <c r="B1784" s="0">
+        <v>116.28360000000001</v>
+      </c>
+      <c r="C1784" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1784" s="0">
+        <v>0.86224742241812402</v>
+      </c>
+    </row>
+    <row r="1785">
+      <c r="A1785" s="0">
+        <v>37.608600000000003</v>
+      </c>
+      <c r="B1785" s="0">
+        <v>101.32689999999999</v>
+      </c>
+      <c r="C1785" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1785" s="0">
+        <v>0.87134723192355701</v>
+      </c>
+    </row>
+    <row r="1786">
+      <c r="A1786" s="0">
+        <v>37.369999999999998</v>
+      </c>
+      <c r="B1786" s="0">
+        <v>101.18000000000001</v>
+      </c>
+      <c r="C1786" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1786" s="0">
+        <v>0.83629959717625602</v>
+      </c>
+    </row>
+    <row r="1787">
+      <c r="A1787" s="0">
+        <v>26.741399999999999</v>
+      </c>
+      <c r="B1787" s="0">
+        <v>115.0581</v>
+      </c>
+      <c r="C1787" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1787" s="0">
+        <v>0.51991887296427997</v>
+      </c>
+    </row>
+    <row r="1788">
+      <c r="A1788" s="0">
+        <v>49.494399999999999</v>
+      </c>
+      <c r="B1788" s="0">
+        <v>18.5429</v>
+      </c>
+      <c r="C1788" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1788" s="0">
+        <v>0.74210474900203205</v>
+      </c>
+    </row>
+    <row r="1789">
+      <c r="A1789" s="0">
+        <v>49.099600000000002</v>
+      </c>
+      <c r="B1789" s="0">
+        <v>13.3047</v>
+      </c>
+      <c r="C1789" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1789" s="0">
+        <v>0.69869367952569395</v>
+      </c>
+    </row>
+    <row r="1790">
+      <c r="A1790" s="0">
+        <v>51.328200000000002</v>
+      </c>
+      <c r="B1790" s="0">
+        <v>10.367800000000001</v>
+      </c>
+      <c r="C1790" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1790" s="0">
+        <v>0.80130343301266804</v>
+      </c>
+    </row>
+    <row r="1791">
+      <c r="A1791" s="0">
+        <v>51.892200000000003</v>
+      </c>
+      <c r="B1791" s="0">
+        <v>14.0337</v>
+      </c>
+      <c r="C1791" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1791" s="0">
+        <v>0.80726956665236005</v>
+      </c>
+    </row>
+    <row r="1792">
+      <c r="A1792" s="0">
+        <v>55.6905</v>
+      </c>
+      <c r="B1792" s="0">
+        <v>12.191800000000001</v>
+      </c>
+      <c r="C1792" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1792" s="0">
+        <v>0.76259872783345095</v>
+      </c>
+    </row>
+    <row r="1793">
+      <c r="A1793" s="0">
+        <v>36.833599999999997</v>
+      </c>
+      <c r="B1793" s="0">
+        <v>-2.2523</v>
+      </c>
+      <c r="C1793" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1793" s="0">
+        <v>0.59536548905891995</v>
+      </c>
+    </row>
+    <row r="1794">
+      <c r="A1794" s="0">
+        <v>37.097900000000003</v>
+      </c>
+      <c r="B1794" s="0">
+        <v>-2.9658000000000002</v>
+      </c>
+      <c r="C1794" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1794" s="0">
+        <v>0.56323259584873497</v>
+      </c>
+    </row>
+    <row r="1795">
+      <c r="A1795" s="0">
+        <v>67.997200000000007</v>
+      </c>
+      <c r="B1795" s="0">
+        <v>24.209199999999999</v>
+      </c>
+      <c r="C1795" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1795" s="0">
+        <v>0.68109420363884898</v>
+      </c>
+    </row>
+    <row r="1796">
+      <c r="A1796" s="0">
+        <v>67.362399999999994</v>
+      </c>
+      <c r="B1796" s="0">
+        <v>26.6386</v>
+      </c>
+      <c r="C1796" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1796" s="0">
+        <v>0.79019895736877</v>
+      </c>
+    </row>
+    <row r="1797">
+      <c r="A1797" s="0">
+        <v>43.741300000000003</v>
+      </c>
+      <c r="B1797" s="0">
+        <v>3.5956999999999999</v>
+      </c>
+      <c r="C1797" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1797" s="0">
+        <v>0.75259420517532405</v>
+      </c>
+    </row>
+    <row r="1798">
+      <c r="A1798" s="0">
+        <v>5.2685000000000004</v>
+      </c>
+      <c r="B1798" s="0">
+        <v>-2.6941999999999999</v>
+      </c>
+      <c r="C1798" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1798" s="0">
+        <v>0.49863614398503198</v>
+      </c>
+    </row>
+    <row r="1799">
+      <c r="A1799" s="0">
+        <v>64.130799999999994</v>
+      </c>
+      <c r="B1799" s="0">
+        <v>-51.386099999999999</v>
+      </c>
+      <c r="C1799" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1799" s="0">
+        <v>0.43947392513741201</v>
+      </c>
+    </row>
+    <row r="1800">
+      <c r="A1800" s="0">
+        <v>74.481399999999994</v>
+      </c>
+      <c r="B1800" s="0">
+        <v>-20.554500000000001</v>
+      </c>
+      <c r="C1800" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1800" s="0">
+        <v>0.044088433122951201</v>
+      </c>
+    </row>
+    <row r="1801">
+      <c r="A1801" s="0">
+        <v>74.473299999999995</v>
+      </c>
+      <c r="B1801" s="0">
+        <v>-20.5503</v>
+      </c>
+      <c r="C1801" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1801" s="0">
+        <v>0.17538036391094899</v>
+      </c>
+    </row>
+    <row r="1802">
+      <c r="A1802" s="0">
+        <v>41.849400000000003</v>
+      </c>
+      <c r="B1802" s="0">
+        <v>13.588100000000001</v>
+      </c>
+      <c r="C1802" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1802" s="0">
+        <v>0.47136067530841502</v>
+      </c>
+    </row>
+    <row r="1803">
+      <c r="A1803" s="0">
+        <v>41.705199999999998</v>
+      </c>
+      <c r="B1803" s="0">
+        <v>12.376099999999999</v>
+      </c>
+      <c r="C1803" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1803" s="0">
+        <v>0.48099816723393901</v>
+      </c>
+    </row>
+    <row r="1804">
+      <c r="A1804" s="0">
+        <v>45.9542</v>
+      </c>
+      <c r="B1804" s="0">
+        <v>11.285299999999999</v>
+      </c>
+      <c r="C1804" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1804" s="0">
+        <v>0.89599891250156405</v>
+      </c>
+    </row>
+    <row r="1805">
+      <c r="A1805" s="0">
+        <v>45.200899999999997</v>
+      </c>
+      <c r="B1805" s="0">
+        <v>9.061</v>
+      </c>
+      <c r="C1805" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1805" s="0">
+        <v>0.64109973486605498</v>
+      </c>
+    </row>
+    <row r="1806">
+      <c r="A1806" s="0">
+        <v>42.408099999999998</v>
+      </c>
+      <c r="B1806" s="0">
+        <v>11.93</v>
+      </c>
+      <c r="C1806" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1806" s="0">
+        <v>0.345146796070471</v>
+      </c>
+    </row>
+    <row r="1807">
+      <c r="A1807" s="0">
+        <v>42.390300000000004</v>
+      </c>
+      <c r="B1807" s="0">
+        <v>11.9209</v>
+      </c>
+      <c r="C1807" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1807" s="0">
+        <v>0.72357110833143101</v>
+      </c>
+    </row>
+    <row r="1808">
+      <c r="A1808" s="0">
+        <v>43.727899999999998</v>
+      </c>
+      <c r="B1808" s="0">
+        <v>10.2844</v>
+      </c>
+      <c r="C1808" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1808" s="0">
+        <v>0.69371475292118001</v>
+      </c>
+    </row>
+    <row r="1809">
+      <c r="A1809" s="0">
+        <v>44.386899999999997</v>
+      </c>
+      <c r="B1809" s="0">
+        <v>142.3186</v>
+      </c>
+      <c r="C1809" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1809" s="0">
+        <v>0.79507674619839397</v>
+      </c>
+    </row>
+    <row r="1810">
+      <c r="A1810" s="0">
+        <v>35.261699999999998</v>
+      </c>
+      <c r="B1810" s="0">
+        <v>137.0788</v>
+      </c>
+      <c r="C1810" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1810" s="0">
+        <v>0.57505321244265095</v>
+      </c>
+    </row>
+    <row r="1811">
+      <c r="A1811" s="0">
+        <v>52.240299999999998</v>
+      </c>
+      <c r="B1811" s="0">
+        <v>5.0712999999999999</v>
+      </c>
+      <c r="C1811" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1811" s="0">
+        <v>0.82744811242501104</v>
+      </c>
+    </row>
+    <row r="1812">
+      <c r="A1812" s="0">
+        <v>52.166600000000003</v>
+      </c>
+      <c r="B1812" s="0">
+        <v>5.7435999999999998</v>
+      </c>
+      <c r="C1812" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1812" s="0">
+        <v>0.77034262896309302</v>
+      </c>
+    </row>
+    <row r="1813">
+      <c r="A1813" s="0">
+        <v>68.613</v>
+      </c>
+      <c r="B1813" s="0">
+        <v>161.34139999999999</v>
+      </c>
+      <c r="C1813" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1813" s="0">
+        <v>0.39043527795767602</v>
+      </c>
+    </row>
+    <row r="1814">
+      <c r="A1814" s="0">
+        <v>70.829099999999997</v>
+      </c>
+      <c r="B1814" s="0">
+        <v>147.49430000000001</v>
+      </c>
+      <c r="C1814" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1814" s="0">
+        <v>0.36186225627094998</v>
+      </c>
+    </row>
+    <row r="1815">
+      <c r="A1815" s="0">
+        <v>54.725200000000001</v>
+      </c>
+      <c r="B1815" s="0">
+        <v>90.002200000000002</v>
+      </c>
+      <c r="C1815" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1815" s="0">
+        <v>0.84229281532179501</v>
+      </c>
+    </row>
+    <row r="1816">
+      <c r="A1816" s="0">
+        <v>72.373800000000003</v>
+      </c>
+      <c r="B1816" s="0">
+        <v>126.4958</v>
+      </c>
+      <c r="C1816" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1816" s="0">
+        <v>0.249301406567808</v>
+      </c>
+    </row>
+    <row r="1817">
+      <c r="A1817" s="0">
+        <v>71.594300000000004</v>
+      </c>
+      <c r="B1817" s="0">
+        <v>128.8878</v>
+      </c>
+      <c r="C1817" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1817" s="0">
+        <v>0.64708305972275304</v>
+      </c>
+    </row>
+    <row r="1818">
+      <c r="A1818" s="0">
+        <v>13.2829</v>
+      </c>
+      <c r="B1818" s="0">
+        <v>30.478300000000001</v>
+      </c>
+      <c r="C1818" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1818" s="0">
+        <v>0.81747136744849802</v>
+      </c>
+    </row>
+    <row r="1819">
+      <c r="A1819" s="0">
+        <v>78.186000000000007</v>
+      </c>
+      <c r="B1819" s="0">
+        <v>15.923</v>
+      </c>
+      <c r="C1819" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1819" s="0">
+        <v>-0.037410813802290901</v>
+      </c>
+    </row>
+    <row r="1820">
+      <c r="A1820" s="0">
+        <v>15.402799999999999</v>
+      </c>
+      <c r="B1820" s="0">
+        <v>-15.4322</v>
+      </c>
+      <c r="C1820" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1820" s="0">
+        <v>0.77161636012568902</v>
+      </c>
+    </row>
+    <row r="1821">
+      <c r="A1821" s="0">
+        <v>70.4696</v>
+      </c>
+      <c r="B1821" s="0">
+        <v>-157.40889999999999</v>
+      </c>
+      <c r="C1821" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1821" s="0">
+        <v>0.41159887802339501</v>
+      </c>
+    </row>
+    <row r="1822">
+      <c r="A1822" s="0">
+        <v>41.3658</v>
+      </c>
+      <c r="B1822" s="0">
+        <v>-106.2397</v>
+      </c>
+      <c r="C1822" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1822" s="0">
+        <v>0.68467187645143401</v>
+      </c>
+    </row>
+    <row r="1823">
+      <c r="A1823" s="0">
+        <v>34.2547</v>
+      </c>
+      <c r="B1823" s="0">
+        <v>-89.873500000000007</v>
+      </c>
+      <c r="C1823" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1823" s="0">
+        <v>0.78746019506873</v>
+      </c>
+    </row>
+    <row r="1824">
+      <c r="A1824" s="0">
+        <v>41.840600000000002</v>
+      </c>
+      <c r="B1824" s="0">
+        <v>-88.241</v>
+      </c>
+      <c r="C1824" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1824" s="0">
+        <v>0.72007885685708195</v>
+      </c>
+    </row>
+    <row r="1825">
+      <c r="A1825" s="0">
+        <v>68.486500000000007</v>
+      </c>
+      <c r="B1825" s="0">
+        <v>-155.75030000000001</v>
+      </c>
+      <c r="C1825" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1825" s="0">
+        <v>0.54841770011795099</v>
+      </c>
+    </row>
+    <row r="1826">
+      <c r="A1826" s="0">
+        <v>28.608599999999999</v>
+      </c>
+      <c r="B1826" s="0">
+        <v>-80.671499999999995</v>
+      </c>
+      <c r="C1826" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1826" s="0">
+        <v>0.50567028885454401</v>
+      </c>
+    </row>
+    <row r="1827">
+      <c r="A1827" s="0">
+        <v>46.082700000000003</v>
+      </c>
+      <c r="B1827" s="0">
+        <v>-89.979200000000006</v>
+      </c>
+      <c r="C1827" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1827" s="0">
+        <v>0.86391079809324001</v>
+      </c>
+    </row>
+    <row r="1828">
+      <c r="A1828" s="0">
+        <v>41.554499999999997</v>
+      </c>
+      <c r="B1828" s="0">
+        <v>-83.843800000000002</v>
+      </c>
+      <c r="C1828" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1828" s="0">
+        <v>0.85026333084648797</v>
+      </c>
+    </row>
+    <row r="1829">
+      <c r="A1829" s="0">
+        <v>45.945900000000002</v>
+      </c>
+      <c r="B1829" s="0">
+        <v>-90.272300000000001</v>
+      </c>
+      <c r="C1829" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1829" s="0">
+        <v>0.84272106504135702</v>
+      </c>
+    </row>
+    <row r="1830">
+      <c r="A1830" s="0">
+        <v>65.1237</v>
+      </c>
+      <c r="B1830" s="0">
+        <v>-147.48759999999999</v>
+      </c>
+      <c r="C1830" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1830" s="0">
+        <v>0.81747776362129299</v>
+      </c>
+    </row>
+    <row r="1831">
+      <c r="A1831" s="0">
+        <v>31.821400000000001</v>
+      </c>
+      <c r="B1831" s="0">
+        <v>-110.8661</v>
+      </c>
+      <c r="C1831" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1831" s="0">
+        <v>0.50843644998482396</v>
+      </c>
+    </row>
+    <row r="1832">
+      <c r="A1832" s="0">
+        <v>41.396599999999999</v>
+      </c>
+      <c r="B1832" s="0">
+        <v>-106.80240000000001</v>
+      </c>
+      <c r="C1832" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1832" s="0">
+        <v>0.827183302525069</v>
+      </c>
+    </row>
+    <row r="1833">
+      <c r="A1833" s="0">
+        <v>45.805900000000001</v>
+      </c>
+      <c r="B1833" s="0">
+        <v>-90.079899999999995</v>
+      </c>
+      <c r="C1833" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1833" s="0">
+        <v>0.87500413137475297</v>
+      </c>
+    </row>
+    <row r="1834">
+      <c r="A1834" s="0">
+        <v>41.464599999999997</v>
+      </c>
+      <c r="B1834" s="0">
+        <v>-82.996200000000002</v>
+      </c>
+      <c r="C1834" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1834" s="0">
+        <v>0.68112821970590498</v>
+      </c>
+    </row>
+    <row r="1835">
+      <c r="A1835" s="0">
+        <v>46.634700000000002</v>
+      </c>
+      <c r="B1835" s="0">
+        <v>-91.098699999999994</v>
+      </c>
+      <c r="C1835" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1835" s="0">
+        <v>0.727575467354308</v>
+      </c>
+    </row>
+    <row r="1836">
+      <c r="A1836" s="0">
+        <v>46.7393</v>
+      </c>
+      <c r="B1836" s="0">
+        <v>-91.166300000000007</v>
+      </c>
+      <c r="C1836" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1836" s="0">
+        <v>0.77093822244274402</v>
+      </c>
+    </row>
+    <row r="1837">
+      <c r="A1837" s="0">
+        <v>-25.0197</v>
+      </c>
+      <c r="B1837" s="0">
+        <v>31.4969</v>
+      </c>
+      <c r="C1837" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1837" s="0">
+        <v>0.65791519434928403</v>
+      </c>
+    </row>
+    <row r="1838">
+      <c r="A1838" s="0">
+        <v>-15.4391</v>
+      </c>
+      <c r="B1838" s="0">
+        <v>23.252500000000001</v>
+      </c>
+      <c r="C1838" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1838" s="0">
+        <v>0.63692221285724005</v>
+      </c>
+    </row>
+    <row r="1839">
+      <c r="A1839" s="0">
+        <v>47.933</v>
+      </c>
+      <c r="B1839" s="0">
+        <v>7.5980999999999996</v>
+      </c>
+      <c r="C1839" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1839" s="0">
+        <v>0.81869168808896398</v>
+      </c>
+    </row>
+    <row r="1840">
+      <c r="A1840" s="0">
+        <v>47.809181000000002</v>
+      </c>
+      <c r="B1840" s="0">
+        <v>11.456168</v>
+      </c>
+      <c r="C1840" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1840" s="0">
+        <v>0.69481742498851495</v>
+      </c>
+    </row>
+    <row r="1841">
+      <c r="A1841" s="0">
+        <v>55.912730000000003</v>
+      </c>
+      <c r="B1841" s="0">
+        <v>8.4048099999999995</v>
+      </c>
+      <c r="C1841" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1841" s="0">
+        <v>0.792014201861729</v>
+      </c>
+    </row>
+    <row r="1842">
+      <c r="A1842" s="0">
+        <v>48.118400000000001</v>
+      </c>
+      <c r="B1842" s="0">
+        <v>-1.7963499999999999</v>
+      </c>
+      <c r="C1842" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1842" s="0">
+        <v>0.62797220774122797</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>